<commit_message>
Added scripts and structural changes
</commit_message>
<xml_diff>
--- a/outputs/evaluation/requirement/validation/gemini-3-1-flash-lite/CF_M04/CF_M04_req_eval_avg.xlsx
+++ b/outputs/evaluation/requirement/validation/gemini-3-1-flash-lite/CF_M04/CF_M04_req_eval_avg.xlsx
@@ -508,6 +508,8 @@
         <v>0.75</v>
       </c>
     </row>
+    <row r="10"/>
+    <row r="11"/>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
@@ -554,6 +556,8 @@
         <v>0.9675</v>
       </c>
     </row>
+    <row r="14"/>
+    <row r="15"/>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
@@ -624,10 +628,8 @@
           <t>fixes</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="B22" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>